<commit_message>
excel iterative pipeline (clean)
</commit_message>
<xml_diff>
--- a/mcp-server/official_server/excel_executor/test_space/test.xlsx
+++ b/mcp-server/official_server/excel_executor/test_space/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\startup\projects\Useit_MCP\mcp-server\official_server\excel_executor\test_space\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE6DF1AA-6AF2-4216-8748-9F573EEBF1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62CAF45-5B65-4D2A-A01A-33E73262C389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="21">
   <si>
     <t>桩号m</t>
   </si>
@@ -104,13 +104,6 @@
     <t>渠底</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
-  <si>
-    <t>跌水2.2</t>
-  </si>
-  <si>
-    <t>接消力池</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
 </sst>
 </file>
 
@@ -135,7 +128,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -145,24 +138,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -179,14 +154,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -467,13 +438,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K26"/>
+  <dimension ref="B1:K24"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -491,7 +459,7 @@
       </c>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -527,7 +495,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -538,11 +506,11 @@
         <v>1730.0229999999999</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E17" si="1">ROUND(D3,2)</f>
+        <f t="shared" ref="E3:E16" si="1">ROUND(D3,2)</f>
         <v>1730.02</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F17" si="2">"1/"&amp;ROUND(1/K3,0)</f>
+        <f t="shared" ref="F3:F16" si="2">"1/"&amp;ROUND(1/K3,0)</f>
         <v>1/100</v>
       </c>
       <c r="G3">
@@ -553,7 +521,7 @@
         <v>1730.16</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I26" si="3">G3-H3</f>
+        <f t="shared" ref="I3:I24" si="3">G3-H3</f>
         <v>0</v>
       </c>
       <c r="J3" s="1">
@@ -564,7 +532,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -601,10 +569,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -619,8 +584,8 @@
         <v>1729.71</v>
       </c>
       <c r="F5" t="str">
-        <f>"1/"&amp;ROUND(1/K5,0)</f>
-        <v>1/200</v>
+        <f t="shared" si="2"/>
+        <v>1/100</v>
       </c>
       <c r="G5">
         <f>E4-K4*(C5-C4)</f>
@@ -638,11 +603,11 @@
         <v>-0.22000000000002728</v>
       </c>
       <c r="K5">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B6" s="3" t="s">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2">
@@ -657,7 +622,7 @@
       </c>
       <c r="F6" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G6">
         <v>1728</v>
@@ -674,10 +639,10 @@
         <v>1.5799999999999272</v>
       </c>
       <c r="K6">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>7</v>
       </c>
@@ -693,28 +658,28 @@
       </c>
       <c r="F7" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G7">
-        <f t="shared" ref="G7:G15" si="4">ROUND(G6-(C7-C6)*K6,2)</f>
-        <v>1727.95</v>
+        <f t="shared" ref="G7:G16" si="4">ROUND(G6-(C7-C6)*K6,2)</f>
+        <v>1727.9</v>
       </c>
       <c r="H7">
         <v>1727.98</v>
       </c>
       <c r="I7">
         <f t="shared" si="3"/>
-        <v>-2.9999999999972715E-2</v>
+        <v>-7.999999999992724E-2</v>
       </c>
       <c r="J7" s="1">
         <f t="shared" si="0"/>
-        <v>1.3499999999999091</v>
+        <v>1.3999999999998636</v>
       </c>
       <c r="K7">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>8</v>
       </c>
@@ -730,28 +695,28 @@
       </c>
       <c r="F8" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G8">
         <f t="shared" si="4"/>
-        <v>1727.9</v>
+        <v>1727.8</v>
       </c>
       <c r="H8">
         <v>1727.96</v>
       </c>
       <c r="I8">
         <f t="shared" si="3"/>
-        <v>-5.999999999994543E-2</v>
+        <v>-0.16000000000008185</v>
       </c>
       <c r="J8" s="1">
         <f>E8-G8</f>
-        <v>1</v>
+        <v>1.1000000000001364</v>
       </c>
       <c r="K8">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>9</v>
       </c>
@@ -767,27 +732,28 @@
       </c>
       <c r="F9" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G9">
         <f t="shared" si="4"/>
-        <v>1727.65</v>
+        <v>1727.3</v>
       </c>
       <c r="H9">
         <v>1727.86</v>
       </c>
       <c r="I9">
         <f t="shared" si="3"/>
-        <v>-0.20999999999980901</v>
+        <v>-0.55999999999994543</v>
       </c>
       <c r="J9" s="1">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>2.4300000000000637</v>
       </c>
       <c r="K9">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>10</v>
       </c>
@@ -803,28 +769,28 @@
       </c>
       <c r="F10" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G10">
         <f t="shared" si="4"/>
-        <v>1727.4</v>
+        <v>1726.8</v>
       </c>
       <c r="H10">
         <v>1727.76</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
-        <v>-0.35999999999989996</v>
+        <v>-0.96000000000003638</v>
       </c>
       <c r="J10" s="1">
         <f t="shared" si="0"/>
-        <v>1.3099999999999454</v>
+        <v>1.9100000000000819</v>
       </c>
       <c r="K10">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>11</v>
       </c>
@@ -840,29 +806,29 @@
       </c>
       <c r="F11" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G11">
         <f t="shared" si="4"/>
-        <v>1727.15</v>
+        <v>1726.3</v>
       </c>
       <c r="H11">
         <v>1727.66</v>
       </c>
       <c r="I11">
         <f t="shared" si="3"/>
-        <v>-0.50999999999999091</v>
+        <v>-1.3600000000001273</v>
       </c>
       <c r="J11" s="1">
         <f t="shared" si="0"/>
-        <v>0.74000000000000909</v>
+        <v>1.5900000000001455</v>
       </c>
       <c r="K11">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B12" s="1" t="s">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2">
@@ -877,29 +843,28 @@
       </c>
       <c r="F12" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G12">
         <f>ROUND(G11-(C12-C11)*K11,2)</f>
-        <v>1727.1</v>
+        <v>1726.2</v>
       </c>
       <c r="H12">
         <v>1727.64</v>
       </c>
       <c r="I12">
         <f t="shared" si="3"/>
-        <v>-0.54000000000019099</v>
+        <v>-1.4400000000000546</v>
       </c>
       <c r="J12" s="1">
-        <f t="shared" ref="J12:J16" si="5">E12-G12</f>
-        <v>0.63000000000010914</v>
+        <f>E12-G12</f>
+        <v>1.5299999999999727</v>
       </c>
       <c r="K12">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B13" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C13" s="2">
         <v>250</v>
       </c>
@@ -913,29 +878,28 @@
       </c>
       <c r="F13" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G13">
         <f>ROUND(G11-(C13-C11)*K11,2)</f>
-        <v>1726.9</v>
+        <v>1725.8</v>
       </c>
       <c r="H13">
         <v>1727.56</v>
       </c>
       <c r="I13">
         <f t="shared" si="3"/>
-        <v>-0.65999999999985448</v>
+        <v>-1.7599999999999909</v>
       </c>
       <c r="J13" s="1">
-        <f t="shared" si="5"/>
-        <v>0.28999999999996362</v>
+        <f>E13-G13</f>
+        <v>1.3900000000001</v>
       </c>
       <c r="K13">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B14" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C14" s="2">
         <v>300</v>
       </c>
@@ -949,32 +913,28 @@
       </c>
       <c r="F14" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>1726.65</v>
+        <v>1725.3</v>
       </c>
       <c r="H14">
         <v>1727.46</v>
       </c>
       <c r="I14">
         <f t="shared" si="3"/>
-        <v>-0.80999999999994543</v>
+        <v>-2.1600000000000819</v>
       </c>
       <c r="J14" s="1">
-        <f t="shared" si="5"/>
-        <v>-0.16000000000008185</v>
+        <f>E14-G14</f>
+        <v>1.1900000000000546</v>
       </c>
       <c r="K14">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C15" s="2">
         <v>350</v>
       </c>
@@ -988,412 +948,343 @@
       </c>
       <c r="F15" t="str">
         <f t="shared" si="2"/>
-        <v>1/200</v>
+        <v>1/100</v>
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>1726.4</v>
+        <v>1724.8</v>
       </c>
       <c r="H15">
         <v>1727.36</v>
       </c>
       <c r="I15">
         <f t="shared" si="3"/>
-        <v>-0.95999999999980901</v>
+        <v>-2.5599999999999454</v>
       </c>
       <c r="J15" s="1">
-        <v>0</v>
+        <f>E15-G15</f>
+        <v>0.99000000000000909</v>
       </c>
       <c r="K15">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B16" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C16" s="2">
-        <f>C15+3</f>
-        <v>353</v>
+        <v>400</v>
       </c>
       <c r="D16">
         <f>D14-0.014*(C16-C14)</f>
-        <v>1725.7429999999999</v>
+        <v>1725.0849999999998</v>
       </c>
       <c r="E16">
-        <f t="shared" ref="E16" si="6">ROUND(D16,2)</f>
-        <v>1725.74</v>
-      </c>
-      <c r="F16" t="str">
-        <f t="shared" ref="F16" si="7">"1/"&amp;ROUND(1/K16,0)</f>
-        <v>1/200</v>
-      </c>
-      <c r="G16">
-        <f>G15-2.2</f>
-        <v>1724.2</v>
-      </c>
-      <c r="H16">
-        <v>1727.36</v>
-      </c>
-      <c r="I16">
-        <f t="shared" ref="I16" si="8">G16-H16</f>
-        <v>-3.1599999999998545</v>
-      </c>
-      <c r="J16" s="1">
-        <f t="shared" si="5"/>
-        <v>1.5399999999999636</v>
-      </c>
-      <c r="K16">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B17" s="4"/>
-      <c r="C17" s="2">
-        <v>400</v>
-      </c>
-      <c r="D17">
-        <f>D14-0.014*(C17-C14)</f>
-        <v>1725.0849999999998</v>
-      </c>
-      <c r="E17">
         <f t="shared" si="1"/>
         <v>1725.09</v>
       </c>
-      <c r="F17" t="str">
-        <f t="shared" si="2"/>
-        <v>1/200</v>
+      <c r="F16" t="str">
+        <f t="shared" si="2"/>
+        <v>1/100</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="4"/>
+        <v>1724.3</v>
+      </c>
+      <c r="H16">
+        <v>1727.26</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>-2.9600000000000364</v>
+      </c>
+      <c r="J16" s="1">
+        <f>E16-G16</f>
+        <v>0.78999999999996362</v>
+      </c>
+      <c r="K16">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="C17" s="2">
+        <v>420</v>
+      </c>
+      <c r="D17">
+        <f t="shared" ref="D17:D18" si="5">D15-0.014*(C17-C15)</f>
+        <v>1724.8049999999998</v>
+      </c>
+      <c r="E17">
+        <f>ROUND(D17,2)</f>
+        <v>1724.81</v>
       </c>
       <c r="G17">
-        <f>ROUND(G15-(C17-C15)*K15,2)</f>
-        <v>1726.15</v>
+        <f>ROUND(G16-(C17-C16)*K16,2)</f>
+        <v>1724.1</v>
       </c>
       <c r="H17">
-        <v>1727.26</v>
+        <v>1727.22</v>
       </c>
       <c r="I17">
         <f t="shared" si="3"/>
-        <v>-1.1099999999999</v>
+        <v>-3.1200000000001182</v>
       </c>
       <c r="J17" s="1">
-        <v>0</v>
+        <f t="shared" ref="J17:J24" si="6">E17-G17</f>
+        <v>0.71000000000003638</v>
       </c>
       <c r="K17">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C18" s="2">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D18">
-        <f>D15-0.014*(C18-C15)</f>
-        <v>1724.8049999999998</v>
+        <f t="shared" si="5"/>
+        <v>1724.7629999999999</v>
       </c>
       <c r="E18">
         <f>ROUND(D18,2)</f>
-        <v>1724.81</v>
+        <v>1724.76</v>
       </c>
       <c r="G18">
-        <f>ROUND(G17-(C18-C17)*K17,2)</f>
-        <v>1726.05</v>
+        <f>G17-2.2</f>
+        <v>1721.8999999999999</v>
       </c>
       <c r="H18">
-        <v>1727.22</v>
+        <v>1725.02</v>
       </c>
       <c r="I18">
         <f t="shared" si="3"/>
-        <v>-1.1700000000000728</v>
+        <v>-3.1200000000001182</v>
       </c>
       <c r="J18" s="1">
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>2.8600000000001273</v>
       </c>
       <c r="K18">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B19" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C19" s="2">
-        <f>C18+3</f>
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="D19">
-        <v>1724.8049999999998</v>
+        <f>D15-0.014*(C19-C15)</f>
+        <v>1724.665</v>
       </c>
       <c r="E19">
-        <v>1724.81</v>
+        <f t="shared" ref="E19:E24" si="7">ROUND(D19,2)</f>
+        <v>1724.67</v>
+      </c>
+      <c r="F19" t="str">
+        <f t="shared" ref="F19:F24" si="8">"1/"&amp;ROUND(1/K19,0)</f>
+        <v>1/100</v>
       </c>
       <c r="G19">
-        <f>G18-2.2</f>
-        <v>1723.85</v>
+        <f>ROUND(G18-(C19-C18-5)*K18,2)</f>
+        <v>1721.88</v>
       </c>
       <c r="H19">
-        <v>1727.22</v>
+        <v>1725.02</v>
       </c>
       <c r="I19">
-        <v>-1.1700000000000728</v>
+        <f t="shared" si="3"/>
+        <v>-3.1399999999998727</v>
       </c>
       <c r="J19" s="1">
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>2.7899999999999636</v>
       </c>
       <c r="K19">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B20" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
       <c r="C20" s="2">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="D20">
-        <f t="shared" ref="D20" si="9">D17-0.014*(C20-C17)</f>
-        <v>1724.7629999999999</v>
+        <f>D16-0.014*(C20-C16)</f>
+        <v>1724.2449999999999</v>
       </c>
       <c r="E20">
-        <f>ROUND(D20,2)</f>
-        <v>1724.76</v>
+        <f t="shared" si="7"/>
+        <v>1724.25</v>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="8"/>
+        <v>1/100</v>
       </c>
       <c r="G20">
-        <f>G18-2.2</f>
-        <v>1723.85</v>
+        <f t="shared" ref="G20:G24" si="9">ROUND(G19-(C20-C19)*K19,2)</f>
+        <v>1721.58</v>
       </c>
       <c r="H20">
-        <v>1725.02</v>
+        <v>1724.96</v>
       </c>
       <c r="I20">
         <f t="shared" si="3"/>
-        <v>-1.1700000000000728</v>
+        <v>-3.3800000000001091</v>
       </c>
       <c r="J20" s="1">
-        <f t="shared" ref="J20:J25" si="10">E20-G20</f>
-        <v>0.91000000000008185</v>
+        <f t="shared" si="6"/>
+        <v>2.6700000000000728</v>
       </c>
       <c r="K20">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B21" s="4"/>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
       <c r="C21" s="2">
-        <v>430</v>
+        <v>464</v>
       </c>
       <c r="D21">
-        <f>D15-0.014*(C21-C15)</f>
-        <v>1724.665</v>
+        <v>1724.03</v>
       </c>
       <c r="E21">
-        <f t="shared" ref="E21:E26" si="11">ROUND(D21,2)</f>
-        <v>1724.67</v>
+        <f t="shared" si="7"/>
+        <v>1724.03</v>
       </c>
       <c r="F21" t="str">
-        <f t="shared" ref="F21:F26" si="12">"1/"&amp;ROUND(1/K21,0)</f>
-        <v>1/200</v>
+        <f t="shared" si="8"/>
+        <v>1/100</v>
       </c>
       <c r="G21">
-        <f>ROUND(G20-(C21-C20-5)*K20,2)</f>
-        <v>1723.84</v>
+        <f t="shared" si="9"/>
+        <v>1721.54</v>
       </c>
       <c r="H21">
-        <v>1725.02</v>
+        <v>1724.95</v>
       </c>
       <c r="I21">
         <f t="shared" si="3"/>
-        <v>-1.1800000000000637</v>
+        <v>-3.4100000000000819</v>
       </c>
       <c r="J21" s="1">
-        <f t="shared" si="10"/>
-        <v>0.83000000000015461</v>
+        <f t="shared" si="6"/>
+        <v>2.4900000000000091</v>
       </c>
       <c r="K21">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B22" s="4" t="s">
-        <v>13</v>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>15</v>
       </c>
       <c r="C22" s="2">
-        <v>460</v>
+        <v>500</v>
       </c>
       <c r="D22">
-        <f>D17-0.014*(C22-C17)</f>
-        <v>1724.2449999999999</v>
+        <v>1723.4590000000001</v>
       </c>
       <c r="E22">
-        <f t="shared" si="11"/>
-        <v>1724.25</v>
+        <f t="shared" si="7"/>
+        <v>1723.46</v>
       </c>
       <c r="F22" t="str">
-        <f t="shared" si="12"/>
-        <v>1/200</v>
+        <f t="shared" si="8"/>
+        <v>1/100</v>
       </c>
       <c r="G22">
-        <f t="shared" ref="G22:G26" si="13">ROUND(G21-(C22-C21)*K21,2)</f>
-        <v>1723.69</v>
+        <f t="shared" si="9"/>
+        <v>1721.18</v>
       </c>
       <c r="H22">
-        <v>1724.96</v>
+        <v>1724.88</v>
       </c>
       <c r="I22">
         <f t="shared" si="3"/>
-        <v>-1.2699999999999818</v>
+        <v>-3.7000000000000455</v>
       </c>
       <c r="J22" s="1">
-        <f t="shared" si="10"/>
-        <v>0.55999999999994543</v>
+        <f t="shared" si="6"/>
+        <v>2.2799999999999727</v>
       </c>
       <c r="K22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B23" s="5" t="s">
-        <v>14</v>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>16</v>
       </c>
       <c r="C23" s="2">
-        <v>464</v>
+        <v>550</v>
       </c>
       <c r="D23">
-        <v>1724.03</v>
+        <v>1722.885</v>
       </c>
       <c r="E23">
-        <f t="shared" si="11"/>
-        <v>1724.03</v>
+        <f t="shared" si="7"/>
+        <v>1722.89</v>
       </c>
       <c r="F23" t="str">
-        <f t="shared" si="12"/>
-        <v>1/200</v>
+        <f t="shared" si="8"/>
+        <v>1/100</v>
       </c>
       <c r="G23">
-        <f t="shared" si="13"/>
-        <v>1723.67</v>
+        <f t="shared" si="9"/>
+        <v>1720.68</v>
       </c>
       <c r="H23">
-        <v>1724.95</v>
+        <v>1724.78</v>
       </c>
       <c r="I23">
         <f t="shared" si="3"/>
-        <v>-1.2799999999999727</v>
+        <v>-4.0999999999999091</v>
       </c>
       <c r="J23" s="1">
-        <f t="shared" si="10"/>
-        <v>0.35999999999989996</v>
+        <f t="shared" si="6"/>
+        <v>2.2100000000000364</v>
       </c>
       <c r="K23">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C24" s="2">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="D24">
-        <v>1723.4590000000001</v>
+        <v>1722.3789999999999</v>
       </c>
       <c r="E24">
-        <f t="shared" si="11"/>
-        <v>1723.46</v>
+        <f t="shared" si="7"/>
+        <v>1722.38</v>
       </c>
       <c r="F24" t="str">
-        <f t="shared" si="12"/>
-        <v>1/200</v>
+        <f t="shared" si="8"/>
+        <v>1/100</v>
       </c>
       <c r="G24">
-        <f t="shared" si="13"/>
-        <v>1723.49</v>
+        <f t="shared" si="9"/>
+        <v>1720.18</v>
       </c>
       <c r="H24">
-        <v>1724.88</v>
+        <v>1724.68</v>
       </c>
       <c r="I24">
         <f t="shared" si="3"/>
-        <v>-1.3900000000001</v>
+        <v>-4.5</v>
       </c>
       <c r="J24" s="1">
-        <f t="shared" si="10"/>
-        <v>-2.9999999999972715E-2</v>
+        <f t="shared" si="6"/>
+        <v>2.2000000000000455</v>
       </c>
       <c r="K24">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="2">
-        <v>550</v>
-      </c>
-      <c r="D25">
-        <v>1722.885</v>
-      </c>
-      <c r="E25">
-        <f t="shared" si="11"/>
-        <v>1722.89</v>
-      </c>
-      <c r="F25" t="str">
-        <f t="shared" si="12"/>
-        <v>1/200</v>
-      </c>
-      <c r="G25">
-        <f t="shared" si="13"/>
-        <v>1723.24</v>
-      </c>
-      <c r="H25">
-        <v>1724.78</v>
-      </c>
-      <c r="I25">
-        <f t="shared" si="3"/>
-        <v>-1.5399999999999636</v>
-      </c>
-      <c r="J25" s="1">
-        <f t="shared" si="10"/>
-        <v>-0.34999999999990905</v>
-      </c>
-      <c r="K25">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="2">
-        <v>600</v>
-      </c>
-      <c r="D26">
-        <v>1722.3789999999999</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="11"/>
-        <v>1722.38</v>
-      </c>
-      <c r="F26" t="str">
-        <f t="shared" si="12"/>
-        <v>1/200</v>
-      </c>
-      <c r="G26">
-        <f t="shared" si="13"/>
-        <v>1722.99</v>
-      </c>
-      <c r="H26">
-        <v>1724.68</v>
-      </c>
-      <c r="I26">
-        <f t="shared" si="3"/>
-        <v>-1.6900000000000546</v>
-      </c>
-      <c r="J26" s="1">
-        <v>0</v>
-      </c>
-      <c r="K26">
-        <v>5.0000000000000001E-3</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -1407,12 +1298,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D01CA33-8443-4FD3-95E1-4429C4922951}">
   <dimension ref="B1:K24"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="9.140625" style="6"/>
-  </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B1" s="6" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
@@ -1430,7 +1318,7 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B2" s="6" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2">
@@ -1466,7 +1354,7 @@
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2">
@@ -1503,7 +1391,7 @@
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="2">
@@ -1540,7 +1428,7 @@
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2">
@@ -1577,7 +1465,7 @@
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2">
@@ -1613,7 +1501,7 @@
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2">
@@ -1650,7 +1538,7 @@
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B8" s="6" t="s">
+      <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2">
@@ -1687,7 +1575,7 @@
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="2">
@@ -1724,7 +1612,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2">
@@ -1761,7 +1649,7 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="2">
@@ -1798,7 +1686,7 @@
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B12" s="6" t="s">
+      <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2">
@@ -2072,7 +1960,7 @@
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B20" s="6" t="s">
+      <c r="B20" t="s">
         <v>13</v>
       </c>
       <c r="C20" s="2">
@@ -2110,7 +1998,7 @@
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B21" s="6" t="s">
+      <c r="B21" t="s">
         <v>14</v>
       </c>
       <c r="C21" s="2">
@@ -2147,7 +2035,7 @@
       </c>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B22" s="6" t="s">
+      <c r="B22" t="s">
         <v>15</v>
       </c>
       <c r="C22" s="2">
@@ -2184,7 +2072,7 @@
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B23" s="6" t="s">
+      <c r="B23" t="s">
         <v>16</v>
       </c>
       <c r="C23" s="2">
@@ -2221,7 +2109,7 @@
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B24" s="6" t="s">
+      <c r="B24" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="2">

</xml_diff>

<commit_message>
add readme, delete unnessary powershell template
</commit_message>
<xml_diff>
--- a/mcp-server/official_server/excel_executor/test_space/test.xlsx
+++ b/mcp-server/official_server/excel_executor/test_space/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\startup\projects\Useit_MCP\mcp-server\official_server\excel_executor\test_space\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62CAF45-5B65-4D2A-A01A-33E73262C389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24264029-B4DC-46BE-9280-618642225232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -510,7 +510,7 @@
         <v>1730.02</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F16" si="2">"1/"&amp;ROUND(1/K3,0)</f>
+        <f t="shared" ref="F3:F18" si="2">"1/"&amp;ROUND(1/K3,0)</f>
         <v>1/100</v>
       </c>
       <c r="G3">
@@ -1016,6 +1016,10 @@
         <f>ROUND(D17,2)</f>
         <v>1724.81</v>
       </c>
+      <c r="F17" t="str">
+        <f t="shared" si="2"/>
+        <v>1/100</v>
+      </c>
       <c r="G17">
         <f>ROUND(G16-(C17-C16)*K16,2)</f>
         <v>1724.1</v>
@@ -1046,6 +1050,10 @@
       <c r="E18">
         <f>ROUND(D18,2)</f>
         <v>1724.76</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="2"/>
+        <v>1/100</v>
       </c>
       <c r="G18">
         <f>G17-2.2</f>
@@ -1368,7 +1376,7 @@
         <v>1730.02</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F16" si="2">"1/"&amp;ROUND(1/K3,0)</f>
+        <f t="shared" ref="F3:F18" si="2">"1/"&amp;ROUND(1/K3,0)</f>
         <v>1/100</v>
       </c>
       <c r="G3">
@@ -1874,6 +1882,10 @@
         <f>ROUND(D17,2)</f>
         <v>1724.81</v>
       </c>
+      <c r="F17" t="str">
+        <f t="shared" si="2"/>
+        <v>1/100</v>
+      </c>
       <c r="G17">
         <f>ROUND(G16-(C17-C16)*K16,2)</f>
         <v>1724.1</v>
@@ -1904,6 +1916,10 @@
       <c r="E18">
         <f>ROUND(D18,2)</f>
         <v>1724.76</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="2"/>
+        <v>1/100</v>
       </c>
       <c r="G18">
         <f>G17-2.2</f>

</xml_diff>